<commit_message>
ci: add fastapi to CI install — worker/app.py imports it at module scope
The @modal.fastapi_endpoint decorator on the trigger() function requires
fastapi at import time, and the test suite triggers that import via
`from app import GOALS_RESPONSE_SCHEMA, ...`. Without fastapi in the CI
env, the regression suite failed at module import.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/ground-truth/judah-2026-05-16-oufc-sosc.xlsx
+++ b/scripts/ground-truth/judah-2026-05-16-oufc-sosc.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="122">
   <si>
     <t>STIX Match Ground-Truth Tagger</t>
   </si>
@@ -143,6 +143,9 @@
     <t>Venue</t>
   </si>
   <si>
+    <t>Home</t>
+  </si>
+  <si>
     <t>Session type</t>
   </si>
   <si>
@@ -152,13 +155,22 @@
     <t>My team color</t>
   </si>
   <si>
+    <t>black</t>
+  </si>
+  <si>
     <t>Outfield jersey colour, lowercase</t>
   </si>
   <si>
     <t>Opponent color</t>
   </si>
   <si>
+    <t>maroon</t>
+  </si>
+  <si>
     <t>My GK color</t>
+  </si>
+  <si>
+    <t>orange</t>
   </si>
   <si>
     <t>Age group</t>
@@ -1025,55 +1037,55 @@
         <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>1</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B7" t="s">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="C7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>1</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B9" t="s">
-        <v>1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B10" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>1</v>
@@ -1081,7 +1093,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B12">
         <v>2</v>
@@ -1089,7 +1101,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -1097,13 +1109,13 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B14" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C14" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -1143,65 +1155,65 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="K1" s="4" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D2" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="I2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C3" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D3" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="I3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
@@ -1874,43 +1886,43 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="N1" s="4" t="s">
         <v>30</v>
@@ -2610,7 +2622,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -2620,7 +2632,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -2628,10 +2640,9 @@
       <c r="E2" s="6"/>
       <c r="F2" s="6"/>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B4" t="s">
         <v>1</v>
@@ -2639,7 +2650,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B5" t="s">
         <v>1</v>
@@ -2647,7 +2658,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B6" t="s">
         <v>1</v>
@@ -2655,7 +2666,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B7" t="s">
         <v>1</v>
@@ -2663,7 +2674,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B8" t="s">
         <v>1</v>
@@ -2671,7 +2682,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B9" t="s">
         <v>1</v>
@@ -2679,7 +2690,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B10" t="s">
         <v>1</v>
@@ -2687,7 +2698,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B11" t="s">
         <v>1</v>
@@ -2695,7 +2706,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B12" t="s">
         <v>1</v>
@@ -2703,142 +2714,140 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B13" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25"/>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="K16" s="4" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C17" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="D17" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="E17" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="F17" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="G17" t="s">
+        <v>107</v>
+      </c>
+      <c r="H17" t="s">
+        <v>108</v>
+      </c>
+      <c r="I17" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C18" t="s">
         <v>103</v>
       </c>
-      <c r="H17" t="s">
+      <c r="D18" t="s">
         <v>104</v>
       </c>
-      <c r="I17" t="s">
+      <c r="E18" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="5" t="s">
+      <c r="F18" t="s">
         <v>106</v>
       </c>
-      <c r="C18" t="s">
-        <v>99</v>
-      </c>
-      <c r="D18" t="s">
-        <v>100</v>
-      </c>
-      <c r="E18" t="s">
-        <v>101</v>
-      </c>
-      <c r="F18" t="s">
-        <v>102</v>
-      </c>
       <c r="H18" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="I18" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="C19" t="s">
+        <v>103</v>
+      </c>
+      <c r="D19" t="s">
+        <v>104</v>
+      </c>
+      <c r="E19" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="5" t="s">
+      <c r="F19" t="s">
+        <v>106</v>
+      </c>
+      <c r="H19" t="s">
         <v>108</v>
       </c>
-      <c r="C19" t="s">
-        <v>99</v>
-      </c>
-      <c r="D19" t="s">
-        <v>100</v>
-      </c>
-      <c r="E19" t="s">
-        <v>101</v>
-      </c>
-      <c r="F19" t="s">
-        <v>102</v>
-      </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C20" t="s">
+        <v>103</v>
+      </c>
+      <c r="D20" t="s">
         <v>104</v>
       </c>
-      <c r="I19" t="s">
+      <c r="E20" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
+      <c r="F20" t="s">
+        <v>106</v>
+      </c>
+      <c r="H20" t="s">
+        <v>111</v>
+      </c>
+      <c r="I20" t="s">
         <v>109</v>
-      </c>
-      <c r="C20" t="s">
-        <v>99</v>
-      </c>
-      <c r="D20" t="s">
-        <v>100</v>
-      </c>
-      <c r="E20" t="s">
-        <v>101</v>
-      </c>
-      <c r="F20" t="s">
-        <v>102</v>
-      </c>
-      <c r="H20" t="s">
-        <v>107</v>
-      </c>
-      <c r="I20" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
@@ -3511,28 +3520,28 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="I1" s="4" t="s">
         <v>30</v>
@@ -4211,25 +4220,25 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>30</v>
@@ -4899,16 +4908,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>30</v>

</xml_diff>